<commit_message>
feat(decision-graph): unify gold-core decisions across intelligence layers
</commit_message>
<xml_diff>
--- a/reports/diagnostics/SENTINEL_RUNTIME_DIAGNOSTICS.xlsx
+++ b/reports/diagnostics/SENTINEL_RUNTIME_DIAGNOSTICS.xlsx
@@ -449,12 +449,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0.9.5.161</t>
+          <t>0.9.5.162</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>v0.9.5.161_report_architecture</t>
+          <t>v0.9.5.162_history_integrity_report_hygiene</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -527,29 +527,29 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>330.196</v>
+        <v>234.262</v>
       </c>
       <c r="B2" t="n">
-        <v>294.105</v>
+        <v>214.913</v>
       </c>
       <c r="C2" t="n">
-        <v>239.907</v>
+        <v>174.003</v>
       </c>
       <c r="D2" t="n">
-        <v>28863.444</v>
+        <v>21771.874</v>
       </c>
       <c r="E2" t="n">
-        <v>558495.291</v>
+        <v>449946.406</v>
       </c>
       <c r="F2" t="n">
-        <v>588228.889</v>
+        <v>472345.044</v>
       </c>
       <c r="G2" t="n">
-        <v>13597.145</v>
+        <v>9554.918</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{'target_rows': 84, 'target_total_ms': 305410.742, 'crop_generation_ms': 3.525, 'variant_build_ms': 225.05, 'ocr_read_ms': 202772.592, 'vote_selection_ms': 7.262, 'avg_target_total_ms': 3635.842, 'slowest_target_ms': 16261.772, 'slowest_target_rank': 23, 'slowest_target_field': 'player_name', 'slowest_target_position': 0}</t>
+          <t>{'target_rows': 84, 'target_total_ms': 222189.853, 'crop_generation_ms': 2.904, 'variant_build_ms': 182.829, 'ocr_read_ms': 148126.082, 'vote_selection_ms': 4.977, 'avg_target_total_ms': 2645.117, 'slowest_target_ms': 12088.911, 'slowest_target_rank': 43, 'slowest_target_field': 'player_name', 'slowest_target_position': 1}</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>330.196</v>
+        <v>234.262</v>
       </c>
     </row>
     <row r="3">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>294.105</v>
+        <v>214.913</v>
       </c>
     </row>
     <row r="4">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>239.907</v>
+        <v>174.003</v>
       </c>
     </row>
     <row r="5">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28863.444</v>
+        <v>21771.874</v>
       </c>
     </row>
     <row r="6">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13597.145</v>
+        <v>9554.918</v>
       </c>
     </row>
     <row r="7">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>588228.889</v>
+        <v>472345.044</v>
       </c>
     </row>
     <row r="8">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>558495.291</v>
+        <v>449946.406</v>
       </c>
     </row>
     <row r="9">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>305410.742</v>
+        <v>222189.853</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3.525</v>
+        <v>2.904</v>
       </c>
     </row>
     <row r="11">
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>225.05</v>
+        <v>182.829</v>
       </c>
     </row>
     <row r="12">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>202772.592</v>
+        <v>148126.082</v>
       </c>
     </row>
     <row r="13">
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7.262</v>
+        <v>4.977</v>
       </c>
     </row>
   </sheetData>
@@ -840,13 +840,13 @@
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>5703.146</v>
+        <v>6034.577</v>
       </c>
       <c r="F2" t="n">
-        <v>5691.156</v>
+        <v>6017.197</v>
       </c>
       <c r="G2" t="n">
-        <v>2851.573</v>
+        <v>3017.288</v>
       </c>
       <c r="H2" t="n">
         <v>4</v>
@@ -872,13 +872,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>11852.886</v>
+        <v>11520.395</v>
       </c>
       <c r="F3" t="n">
-        <v>6333.179</v>
+        <v>6199.076</v>
       </c>
       <c r="G3" t="n">
-        <v>5926.443</v>
+        <v>5760.198</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
@@ -904,13 +904,13 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>11925.347</v>
+        <v>8080.658</v>
       </c>
       <c r="F4" t="n">
-        <v>11903.177</v>
+        <v>8061.709</v>
       </c>
       <c r="G4" t="n">
-        <v>3975.116</v>
+        <v>2693.553</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
@@ -968,13 +968,13 @@
         <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>27631.169</v>
+        <v>19500.769</v>
       </c>
       <c r="F6" t="n">
-        <v>27573.755</v>
+        <v>19450.124</v>
       </c>
       <c r="G6" t="n">
-        <v>3453.896</v>
+        <v>2437.596</v>
       </c>
       <c r="H6" t="n">
         <v>4</v>
@@ -1000,13 +1000,13 @@
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>3443.629</v>
+        <v>2591.022</v>
       </c>
       <c r="F7" t="n">
-        <v>3422.958</v>
+        <v>2581.253</v>
       </c>
       <c r="G7" t="n">
-        <v>1721.814</v>
+        <v>1295.511</v>
       </c>
       <c r="H7" t="n">
         <v>4</v>
@@ -1032,13 +1032,13 @@
         <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>30197.915</v>
+        <v>21853.684</v>
       </c>
       <c r="F8" t="n">
-        <v>15765.29</v>
+        <v>11699</v>
       </c>
       <c r="G8" t="n">
-        <v>3774.739</v>
+        <v>2731.71</v>
       </c>
       <c r="H8" t="n">
         <v>4</v>
@@ -1064,13 +1064,13 @@
         <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.056</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0.042</v>
+        <v>0.028</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -1096,13 +1096,13 @@
         <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>81283.788</v>
+        <v>57585.597</v>
       </c>
       <c r="F10" t="n">
-        <v>63786.397</v>
+        <v>44357.074</v>
       </c>
       <c r="G10" t="n">
-        <v>5418.919</v>
+        <v>3839.04</v>
       </c>
       <c r="H10" t="n">
         <v>4</v>
@@ -1128,13 +1128,13 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>98588.23299999999</v>
+        <v>64756.733</v>
       </c>
       <c r="F11" t="n">
-        <v>44923.168</v>
+        <v>29649.028</v>
       </c>
       <c r="G11" t="n">
-        <v>7042.017</v>
+        <v>4625.481</v>
       </c>
       <c r="H11" t="n">
         <v>4.571</v>
@@ -1160,13 +1160,13 @@
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>34784.545</v>
+        <v>30266.362</v>
       </c>
       <c r="F12" t="n">
-        <v>23373.512</v>
+        <v>20111.621</v>
       </c>
       <c r="G12" t="n">
-        <v>8696.136</v>
+        <v>7566.59</v>
       </c>
       <c r="H12" t="n">
         <v>5</v>

</xml_diff>